<commit_message>
Add explicit scope field to PAC template
</commit_message>
<xml_diff>
--- a/public/templates/PAC-Certification-Template.xlsx
+++ b/public/templates/PAC-Certification-Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main Tracker" sheetId="1" r:id="Rcccbd0ed9dec4f0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Our AP" sheetId="2" r:id="Rf1616b1cf3424d83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main Tracker" sheetId="1" r:id="R9bf4873642754f72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Our AP" sheetId="2" r:id="R4ebcf24d58984fa8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -462,6 +462,7 @@
     <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="30" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="30" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -520,6 +521,9 @@
       </x:c>
       <x:c r="M2" s="24" t="str">
         <x:v>Remarks</x:v>
+      </x:c>
+      <x:c r="N2" s="24" t="str">
+        <x:v>In Scope</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -536,6 +540,9 @@
       <x:c r="K3" s="19"/>
       <x:c r="L3" s="19"/>
       <x:c r="M3" s="26"/>
+      <x:c r="N3" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="25"/>
@@ -551,6 +558,9 @@
       <x:c r="K4" s="19"/>
       <x:c r="L4" s="19"/>
       <x:c r="M4" s="26"/>
+      <x:c r="N4" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="25"/>
@@ -566,6 +576,9 @@
       <x:c r="K5" s="19"/>
       <x:c r="L5" s="19"/>
       <x:c r="M5" s="26"/>
+      <x:c r="N5" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="25"/>
@@ -581,6 +594,9 @@
       <x:c r="K6" s="19"/>
       <x:c r="L6" s="19"/>
       <x:c r="M6" s="26"/>
+      <x:c r="N6" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="25"/>
@@ -596,6 +612,9 @@
       <x:c r="K7" s="19"/>
       <x:c r="L7" s="19"/>
       <x:c r="M7" s="26"/>
+      <x:c r="N7" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="25"/>
@@ -611,6 +630,9 @@
       <x:c r="K8" s="19"/>
       <x:c r="L8" s="19"/>
       <x:c r="M8" s="26"/>
+      <x:c r="N8" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="25"/>
@@ -626,6 +648,9 @@
       <x:c r="K9" s="19"/>
       <x:c r="L9" s="19"/>
       <x:c r="M9" s="26"/>
+      <x:c r="N9" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="25"/>
@@ -641,6 +666,9 @@
       <x:c r="K10" s="19"/>
       <x:c r="L10" s="19"/>
       <x:c r="M10" s="26"/>
+      <x:c r="N10" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="25"/>
@@ -656,6 +684,9 @@
       <x:c r="K11" s="19"/>
       <x:c r="L11" s="19"/>
       <x:c r="M11" s="26"/>
+      <x:c r="N11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="25"/>
@@ -671,6 +702,9 @@
       <x:c r="K12" s="19"/>
       <x:c r="L12" s="19"/>
       <x:c r="M12" s="26"/>
+      <x:c r="N12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="25"/>
@@ -686,6 +720,9 @@
       <x:c r="K13" s="19"/>
       <x:c r="L13" s="19"/>
       <x:c r="M13" s="26"/>
+      <x:c r="N13" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="25"/>
@@ -701,6 +738,9 @@
       <x:c r="K14" s="19"/>
       <x:c r="L14" s="19"/>
       <x:c r="M14" s="26"/>
+      <x:c r="N14" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="25"/>
@@ -716,6 +756,9 @@
       <x:c r="K15" s="19"/>
       <x:c r="L15" s="19"/>
       <x:c r="M15" s="26"/>
+      <x:c r="N15" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="25"/>
@@ -731,6 +774,9 @@
       <x:c r="K16" s="19"/>
       <x:c r="L16" s="19"/>
       <x:c r="M16" s="26"/>
+      <x:c r="N16" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="25"/>
@@ -746,6 +792,9 @@
       <x:c r="K17" s="19"/>
       <x:c r="L17" s="19"/>
       <x:c r="M17" s="26"/>
+      <x:c r="N17" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="25"/>
@@ -761,6 +810,9 @@
       <x:c r="K18" s="19"/>
       <x:c r="L18" s="19"/>
       <x:c r="M18" s="26"/>
+      <x:c r="N18" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="25"/>
@@ -776,6 +828,9 @@
       <x:c r="K19" s="19"/>
       <x:c r="L19" s="19"/>
       <x:c r="M19" s="26"/>
+      <x:c r="N19" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="25"/>
@@ -791,6 +846,9 @@
       <x:c r="K20" s="19"/>
       <x:c r="L20" s="19"/>
       <x:c r="M20" s="26"/>
+      <x:c r="N20" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="25"/>
@@ -806,6 +864,9 @@
       <x:c r="K21" s="19"/>
       <x:c r="L21" s="19"/>
       <x:c r="M21" s="26"/>
+      <x:c r="N21" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="25"/>
@@ -821,6 +882,9 @@
       <x:c r="K22" s="19"/>
       <x:c r="L22" s="19"/>
       <x:c r="M22" s="26"/>
+      <x:c r="N22" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="25"/>
@@ -836,6 +900,9 @@
       <x:c r="K23" s="19"/>
       <x:c r="L23" s="19"/>
       <x:c r="M23" s="26"/>
+      <x:c r="N23" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="25"/>
@@ -851,6 +918,9 @@
       <x:c r="K24" s="19"/>
       <x:c r="L24" s="19"/>
       <x:c r="M24" s="26"/>
+      <x:c r="N24" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="25"/>
@@ -866,6 +936,9 @@
       <x:c r="K25" s="19"/>
       <x:c r="L25" s="19"/>
       <x:c r="M25" s="26"/>
+      <x:c r="N25" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="25"/>
@@ -881,6 +954,9 @@
       <x:c r="K26" s="19"/>
       <x:c r="L26" s="19"/>
       <x:c r="M26" s="26"/>
+      <x:c r="N26" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="25"/>
@@ -896,6 +972,9 @@
       <x:c r="K27" s="19"/>
       <x:c r="L27" s="19"/>
       <x:c r="M27" s="26"/>
+      <x:c r="N27" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="25"/>
@@ -911,6 +990,9 @@
       <x:c r="K28" s="19"/>
       <x:c r="L28" s="19"/>
       <x:c r="M28" s="26"/>
+      <x:c r="N28" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="25"/>
@@ -926,6 +1008,9 @@
       <x:c r="K29" s="19"/>
       <x:c r="L29" s="19"/>
       <x:c r="M29" s="26"/>
+      <x:c r="N29" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="25"/>
@@ -941,6 +1026,9 @@
       <x:c r="K30" s="19"/>
       <x:c r="L30" s="19"/>
       <x:c r="M30" s="26"/>
+      <x:c r="N30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="25"/>
@@ -956,6 +1044,9 @@
       <x:c r="K31" s="19"/>
       <x:c r="L31" s="19"/>
       <x:c r="M31" s="26"/>
+      <x:c r="N31" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="25"/>
@@ -971,6 +1062,9 @@
       <x:c r="K32" s="19"/>
       <x:c r="L32" s="19"/>
       <x:c r="M32" s="26"/>
+      <x:c r="N32" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="25"/>
@@ -986,6 +1080,9 @@
       <x:c r="K33" s="19"/>
       <x:c r="L33" s="19"/>
       <x:c r="M33" s="26"/>
+      <x:c r="N33" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="25"/>
@@ -1001,6 +1098,9 @@
       <x:c r="K34" s="19"/>
       <x:c r="L34" s="19"/>
       <x:c r="M34" s="26"/>
+      <x:c r="N34" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="25"/>
@@ -1016,6 +1116,9 @@
       <x:c r="K35" s="19"/>
       <x:c r="L35" s="19"/>
       <x:c r="M35" s="26"/>
+      <x:c r="N35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="25"/>
@@ -1031,6 +1134,9 @@
       <x:c r="K36" s="19"/>
       <x:c r="L36" s="19"/>
       <x:c r="M36" s="26"/>
+      <x:c r="N36" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="25"/>
@@ -1046,6 +1152,9 @@
       <x:c r="K37" s="19"/>
       <x:c r="L37" s="19"/>
       <x:c r="M37" s="26"/>
+      <x:c r="N37" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="25"/>
@@ -1061,6 +1170,9 @@
       <x:c r="K38" s="19"/>
       <x:c r="L38" s="19"/>
       <x:c r="M38" s="26"/>
+      <x:c r="N38" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="25"/>
@@ -1076,6 +1188,9 @@
       <x:c r="K39" s="19"/>
       <x:c r="L39" s="19"/>
       <x:c r="M39" s="26"/>
+      <x:c r="N39" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="25"/>
@@ -1091,6 +1206,9 @@
       <x:c r="K40" s="19"/>
       <x:c r="L40" s="19"/>
       <x:c r="M40" s="26"/>
+      <x:c r="N40" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="25"/>
@@ -1106,6 +1224,9 @@
       <x:c r="K41" s="19"/>
       <x:c r="L41" s="19"/>
       <x:c r="M41" s="26"/>
+      <x:c r="N41" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="25"/>
@@ -1121,6 +1242,9 @@
       <x:c r="K42" s="19"/>
       <x:c r="L42" s="19"/>
       <x:c r="M42" s="26"/>
+      <x:c r="N42" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="25"/>
@@ -1136,6 +1260,9 @@
       <x:c r="K43" s="19"/>
       <x:c r="L43" s="19"/>
       <x:c r="M43" s="26"/>
+      <x:c r="N43" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="25"/>
@@ -1151,6 +1278,9 @@
       <x:c r="K44" s="19"/>
       <x:c r="L44" s="19"/>
       <x:c r="M44" s="26"/>
+      <x:c r="N44" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="25"/>
@@ -1166,6 +1296,9 @@
       <x:c r="K45" s="19"/>
       <x:c r="L45" s="19"/>
       <x:c r="M45" s="26"/>
+      <x:c r="N45" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="25"/>
@@ -1181,6 +1314,9 @@
       <x:c r="K46" s="19"/>
       <x:c r="L46" s="19"/>
       <x:c r="M46" s="26"/>
+      <x:c r="N46" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="25"/>
@@ -1196,6 +1332,9 @@
       <x:c r="K47" s="19"/>
       <x:c r="L47" s="19"/>
       <x:c r="M47" s="26"/>
+      <x:c r="N47" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="25"/>
@@ -1211,6 +1350,9 @@
       <x:c r="K48" s="19"/>
       <x:c r="L48" s="19"/>
       <x:c r="M48" s="26"/>
+      <x:c r="N48" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="25"/>
@@ -1226,6 +1368,9 @@
       <x:c r="K49" s="19"/>
       <x:c r="L49" s="19"/>
       <x:c r="M49" s="26"/>
+      <x:c r="N49" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="25"/>
@@ -1241,6 +1386,9 @@
       <x:c r="K50" s="19"/>
       <x:c r="L50" s="19"/>
       <x:c r="M50" s="26"/>
+      <x:c r="N50" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="25"/>
@@ -1256,6 +1404,9 @@
       <x:c r="K51" s="19"/>
       <x:c r="L51" s="19"/>
       <x:c r="M51" s="26"/>
+      <x:c r="N51" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="25"/>
@@ -1271,6 +1422,9 @@
       <x:c r="K52" s="19"/>
       <x:c r="L52" s="19"/>
       <x:c r="M52" s="26"/>
+      <x:c r="N52" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="25"/>
@@ -3526,6 +3680,11 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:M1"/>
   </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="N3:N52">
+      <x:formula1>"Yes,No"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>

</xml_diff>